<commit_message>
created basic frontend , including dashboard
</commit_message>
<xml_diff>
--- a/output.xlsx
+++ b/output.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet3" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet3" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,16 +20,13 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -40,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -48,21 +45,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -429,56 +417,56 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J12"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>deposit_slip_no</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>txt_amount</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>txt_station</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>txt_date</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>excel_amount</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>excel_station</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>excel_area</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>excel_date</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>difference</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>state</t>
         </is>
@@ -506,7 +494,7 @@
           <t>AUWA</t>
         </is>
       </c>
-      <c r="H2" s="2" t="n">
+      <c r="H2" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="I2" t="inlineStr"/>
@@ -519,7 +507,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>A04689</t>
+          <t>CBAJIT00CF</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -527,10 +515,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>INAGAR JAIPUR     COMM</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr"/>
+          <t>GANDHINAGAR JAIPUR</t>
+        </is>
+      </c>
+      <c r="D3" s="1" t="n">
+        <v>46098</v>
+      </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr"/>
@@ -545,46 +535,42 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CBXBWA00CC</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="n">
-        <v>250</v>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>BWA</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>BHINWALIYA</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="n">
-        <v>46101</v>
-      </c>
+          <t>CBGADJ00CI</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>492287</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>GANDHINAGAR JAIPUR</t>
+        </is>
+      </c>
+      <c r="D4" s="1" t="n">
+        <v>46098</v>
+      </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr">
         <is>
-          <t>UNMATCHED_EXCEL</t>
+          <t>UNMATCHED_TXT</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CBXBWA00CD</t>
+          <t>CBXBWA00CC</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="n">
-        <v>1100</v>
+        <v>250</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -596,7 +582,7 @@
           <t>BHINWALIYA</t>
         </is>
       </c>
-      <c r="H5" s="2" t="n">
+      <c r="H5" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="I5" t="inlineStr"/>
@@ -609,14 +595,14 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CBXBWA00CE</t>
+          <t>CBXBWA00CD</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="n">
-        <v>460</v>
+        <v>1100</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -628,7 +614,7 @@
           <t>BHINWALIYA</t>
         </is>
       </c>
-      <c r="H6" s="2" t="n">
+      <c r="H6" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="I6" t="inlineStr"/>
@@ -641,14 +627,14 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CBXBWA00CF</t>
+          <t>CBXBWA00CE</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="n">
-        <v>250</v>
+        <v>460</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -660,7 +646,7 @@
           <t>BHINWALIYA</t>
         </is>
       </c>
-      <c r="H7" s="2" t="n">
+      <c r="H7" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="I7" t="inlineStr"/>
@@ -673,26 +659,26 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CBXJAL00CB</t>
+          <t>CBXBWA00CF</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="n">
-        <v>4770</v>
+        <v>250</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>JAL</t>
+          <t>BWA</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>JAWALI</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="n">
+          <t>BHINWALIYA</t>
+        </is>
+      </c>
+      <c r="H8" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="I8" t="inlineStr"/>
@@ -705,14 +691,14 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CBXJAL00CC</t>
+          <t>CBXJAL00CB</t>
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="n">
-        <v>3555</v>
+        <v>4770</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -724,7 +710,7 @@
           <t>JAWALI</t>
         </is>
       </c>
-      <c r="H9" s="2" t="n">
+      <c r="H9" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="I9" t="inlineStr"/>
@@ -737,26 +723,26 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CBXSEU00CE</t>
+          <t>CBXJAL00CC</t>
         </is>
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="n">
-        <v>4425</v>
+        <v>3555</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>SEU</t>
+          <t>JAL</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>SENDRA</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="n">
+          <t>JAWALI</t>
+        </is>
+      </c>
+      <c r="H10" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="I10" t="inlineStr"/>
@@ -769,14 +755,14 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CBXSEU00CF</t>
+          <t>CBXSEU00CE</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="n">
-        <v>3550</v>
+        <v>4425</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -788,7 +774,7 @@
           <t>SENDRA</t>
         </is>
       </c>
-      <c r="H11" s="2" t="n">
+      <c r="H11" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="I11" t="inlineStr"/>
@@ -801,30 +787,62 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CBXXHP00CC</t>
+          <t>CBXSEU00CF</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="n">
-        <v>16225</v>
+        <v>3550</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>SEU</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Haripur</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="n">
+          <t>SENDRA</t>
+        </is>
+      </c>
+      <c r="H12" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr">
+        <is>
+          <t>UNMATCHED_EXCEL</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>CBXXHP00CC</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr"/>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="n">
+        <v>16225</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>HP</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Haripur</t>
+        </is>
+      </c>
+      <c r="H13" s="1" t="n">
+        <v>46101</v>
+      </c>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr">
         <is>
           <t>UNMATCHED_EXCEL</t>
         </is>

</xml_diff>